<commit_message>
Add cards-blog, columns-media blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 50
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-blog-home.report.xlsx
+++ b/tools/importer/reports/import-blog-home.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="535">
   <si>
     <t>_reportFile</t>
   </si>
@@ -349,7 +349,7 @@
     <t>blog-home</t>
   </si>
   <si>
-    <t>2026-10-11T15:20:43.210Z</t>
+    <t>2026-10-11T16:16:44.295Z</t>
   </si>
   <si>
     <t>Blog</t>
@@ -440,6 +440,207 @@
   </si>
   <si>
     <t>https://help.parker.com/us/en/support</t>
+  </si>
+  <si>
+    <t>us/en/blog/comparing-silver-plated-and-nickel-plated-aluminum-emi-shielding-particles.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media"]</t>
+  </si>
+  <si>
+    <t>us/en/blog/comparing-silver-plated-and-nickel-plated-aluminum-emi-shielding-particles</t>
+  </si>
+  <si>
+    <t>blog-article</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:42.179Z</t>
+  </si>
+  <si>
+    <t>Comparing Silver-Plated and Nickel-Plated Aluminum EMI Shielding Particles</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/comparing-silver-plated-and-nickel--plated-aluminum-emi-shielding-particles.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/emi-shielding-and-thermal-management-for-robotics.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media","columns-media","columns-media"]</t>
+  </si>
+  <si>
+    <t>us/en/blog/emi-shielding-and-thermal-management-for-robotics</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:55.942Z</t>
+  </si>
+  <si>
+    <t>EMI Shielding and Thermal Management for Robotics</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/emi-shielding-and-thermal-management-for-robotics.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/emi-shielding-and-thermal-solutions-for-electric-transportation.report.json</t>
+  </si>
+  <si>
+    <t>us/en/blog/emi-shielding-and-thermal-solutions-for-electric-transportation</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:52.773Z</t>
+  </si>
+  <si>
+    <t>EMI Shielding and Thermal Solutions for Electric Transportation</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/emi-shielding-and-thermal-solutions-for-electric-transportation.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/emi-shielding-within-medical-device-applications.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media","columns-media"]</t>
+  </si>
+  <si>
+    <t>us/en/blog/emi-shielding-within-medical-device-applications</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:46.371Z</t>
+  </si>
+  <si>
+    <t>EMI Shielding Within Medical Device Applications</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/emi-shielding-within-medical-device-applications.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/essential-protection-for-high-performance-drone-systems.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media"]</t>
+  </si>
+  <si>
+    <t>us/en/blog/essential-protection-for-high-performance-drone-systems</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:37.529Z</t>
+  </si>
+  <si>
+    <t>EMI Shielding: Essential Protection for High-Performance Drone Systems</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/essential-protection-for-high-performance-drone-systems.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/helping-oems-find-right-hydraulic-cylinder-solution.report.json</t>
+  </si>
+  <si>
+    <t>us/en/blog/helping-oems-find-right-hydraulic-cylinder-solution</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:44.127Z</t>
+  </si>
+  <si>
+    <t>Helping OEMs Find the Right Hydraulic Cylinder Solution</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/msg_grp/helping-oems-find-right-hydraulic-cylinder-solution.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/how-do-thermal-interface-materials-support-leo-small-satellite-electronics.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media","columns-media","columns-media","columns-media","columns-media"]</t>
+  </si>
+  <si>
+    <t>us/en/blog/how-do-thermal-interface-materials-support-leo-small-satellite-electronics</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:39.554Z</t>
+  </si>
+  <si>
+    <t>How Do Thermal Interface Materials Support Low Earth Orbit Small Satellite Electronics</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/how-do-thermal-interface-materials-support-leo-small-satellite-electronics.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/how-parker-chelsea-helps-oems-fleets-improve-pto-performance.report.json</t>
+  </si>
+  <si>
+    <t>us/en/blog/how-parker-chelsea-helps-oems-fleets-improve-pto-performance</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:58.605Z</t>
+  </si>
+  <si>
+    <t>How Parker Chelsea Helps OEMs and Fleets Improve PTO Performance</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/msg_grp/How-Parker-Chelsea-Helps-OEMs-Fleets-Improve-PTO-Performance.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/radar-across-every-domain.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media","table"]</t>
+  </si>
+  <si>
+    <t>us/en/blog/radar-across-every-domain</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:50.925Z</t>
+  </si>
+  <si>
+    <t>Radar Across Every Domain</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/radar-across-every-domain.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/space-payload-emi-shielding.report.json</t>
+  </si>
+  <si>
+    <t>us/en/blog/space-payload-emi-shielding</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:34.973Z</t>
+  </si>
+  <si>
+    <t>Space Payload EMI Shielding: Conductive Gasket Selection for Payload Enclosures</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/space-payload-emi-shielding.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/thermal-management-for-optical-transceivers.report.json</t>
+  </si>
+  <si>
+    <t>us/en/blog/thermal-management-for-optical-transceivers</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:16:00.662Z</t>
+  </si>
+  <si>
+    <t>Thermal Management for Optical Transceivers</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/thermal-management-for-optical-transceivers.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/why-documentation-and-end-user-insight-matter-in-hydraulic-design.report.json</t>
+  </si>
+  <si>
+    <t>us/en/blog/why-documentation-and-end-user-insight-matter-in-hydraulic-design</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:48.816Z</t>
+  </si>
+  <si>
+    <t>Why Documentation, Collaboration and End-User Insight Matter in Hydraulic Design</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/msg_grp/why-documentation-and-end-user-insight-matter-in-hydraulic-design.html</t>
   </si>
   <si>
     <t>us/en/category/adhesives-coatings-and-encapsulants.report.json</t>
@@ -1805,7 +2006,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J96"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="50" customWidth="1"/>
@@ -2650,7 +2851,7 @@
         <v>150</v>
       </c>
       <c r="B27" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C27" t="s">
         <v>11</v>
@@ -2659,7 +2860,7 @@
         <v>11</v>
       </c>
       <c r="E27" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F27" t="s">
         <v>13</v>
@@ -2668,21 +2869,21 @@
         <v>146</v>
       </c>
       <c r="H27" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I27" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J27" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B28" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C28" t="s">
         <v>11</v>
@@ -2691,7 +2892,7 @@
         <v>11</v>
       </c>
       <c r="E28" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F28" t="s">
         <v>13</v>
@@ -2700,21 +2901,21 @@
         <v>146</v>
       </c>
       <c r="H28" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I28" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J28" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B29" t="s">
-        <v>144</v>
+        <v>162</v>
       </c>
       <c r="C29" t="s">
         <v>11</v>
@@ -2723,7 +2924,7 @@
         <v>11</v>
       </c>
       <c r="E29" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F29" t="s">
         <v>13</v>
@@ -2732,21 +2933,21 @@
         <v>146</v>
       </c>
       <c r="H29" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="I29" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="J29" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B30" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="C30" t="s">
         <v>11</v>
@@ -2755,7 +2956,7 @@
         <v>11</v>
       </c>
       <c r="E30" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="F30" t="s">
         <v>13</v>
@@ -2764,21 +2965,21 @@
         <v>146</v>
       </c>
       <c r="H30" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="I30" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="J30" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B31" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C31" t="s">
         <v>11</v>
@@ -2787,7 +2988,7 @@
         <v>11</v>
       </c>
       <c r="E31" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="F31" t="s">
         <v>13</v>
@@ -2796,21 +2997,21 @@
         <v>146</v>
       </c>
       <c r="H31" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="I31" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="J31" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B32" t="s">
-        <v>144</v>
+        <v>179</v>
       </c>
       <c r="C32" t="s">
         <v>11</v>
@@ -2819,7 +3020,7 @@
         <v>11</v>
       </c>
       <c r="E32" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="F32" t="s">
         <v>13</v>
@@ -2828,21 +3029,21 @@
         <v>146</v>
       </c>
       <c r="H32" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="I32" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="J32" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B33" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C33" t="s">
         <v>11</v>
@@ -2851,7 +3052,7 @@
         <v>11</v>
       </c>
       <c r="E33" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="F33" t="s">
         <v>13</v>
@@ -2860,21 +3061,21 @@
         <v>146</v>
       </c>
       <c r="H33" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="I33" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="J33" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B34" t="s">
-        <v>144</v>
+        <v>190</v>
       </c>
       <c r="C34" t="s">
         <v>11</v>
@@ -2883,7 +3084,7 @@
         <v>11</v>
       </c>
       <c r="E34" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="F34" t="s">
         <v>13</v>
@@ -2892,21 +3093,21 @@
         <v>146</v>
       </c>
       <c r="H34" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="I34" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="J34" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="B35" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C35" t="s">
         <v>11</v>
@@ -2915,7 +3116,7 @@
         <v>11</v>
       </c>
       <c r="E35" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="F35" t="s">
         <v>13</v>
@@ -2924,18 +3125,18 @@
         <v>146</v>
       </c>
       <c r="H35" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="I35" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="J35" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="B36" t="s">
         <v>144</v>
@@ -2947,7 +3148,7 @@
         <v>11</v>
       </c>
       <c r="E36" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="F36" t="s">
         <v>13</v>
@@ -2956,21 +3157,21 @@
         <v>146</v>
       </c>
       <c r="H36" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="I36" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="J36" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="B37" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C37" t="s">
         <v>11</v>
@@ -2979,7 +3180,7 @@
         <v>11</v>
       </c>
       <c r="E37" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="F37" t="s">
         <v>13</v>
@@ -2988,21 +3189,21 @@
         <v>146</v>
       </c>
       <c r="H37" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="I37" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="J37" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="B38" t="s">
-        <v>144</v>
+        <v>211</v>
       </c>
       <c r="C38" t="s">
         <v>11</v>
@@ -3011,30 +3212,30 @@
         <v>11</v>
       </c>
       <c r="E38" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="F38" t="s">
         <v>13</v>
       </c>
       <c r="G38" t="s">
-        <v>146</v>
+        <v>213</v>
       </c>
       <c r="H38" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="I38" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="J38" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="B39" t="s">
-        <v>144</v>
+        <v>211</v>
       </c>
       <c r="C39" t="s">
         <v>11</v>
@@ -3043,30 +3244,30 @@
         <v>11</v>
       </c>
       <c r="E39" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="F39" t="s">
         <v>13</v>
       </c>
       <c r="G39" t="s">
-        <v>146</v>
+        <v>213</v>
       </c>
       <c r="H39" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="I39" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="J39" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="B40" t="s">
-        <v>144</v>
+        <v>211</v>
       </c>
       <c r="C40" t="s">
         <v>11</v>
@@ -3075,30 +3276,30 @@
         <v>11</v>
       </c>
       <c r="E40" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="F40" t="s">
         <v>13</v>
       </c>
       <c r="G40" t="s">
-        <v>146</v>
+        <v>213</v>
       </c>
       <c r="H40" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="I40" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="J40" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="B41" t="s">
-        <v>144</v>
+        <v>211</v>
       </c>
       <c r="C41" t="s">
         <v>11</v>
@@ -3107,30 +3308,30 @@
         <v>11</v>
       </c>
       <c r="E41" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="F41" t="s">
         <v>13</v>
       </c>
       <c r="G41" t="s">
-        <v>146</v>
+        <v>213</v>
       </c>
       <c r="H41" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="I41" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="J41" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="B42" t="s">
-        <v>144</v>
+        <v>211</v>
       </c>
       <c r="C42" t="s">
         <v>11</v>
@@ -3139,30 +3340,30 @@
         <v>11</v>
       </c>
       <c r="E42" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="F42" t="s">
         <v>13</v>
       </c>
       <c r="G42" t="s">
-        <v>146</v>
+        <v>213</v>
       </c>
       <c r="H42" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="I42" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="J42" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="B43" t="s">
-        <v>144</v>
+        <v>211</v>
       </c>
       <c r="C43" t="s">
         <v>11</v>
@@ -3171,30 +3372,30 @@
         <v>11</v>
       </c>
       <c r="E43" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="F43" t="s">
         <v>13</v>
       </c>
       <c r="G43" t="s">
-        <v>146</v>
+        <v>213</v>
       </c>
       <c r="H43" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="I43" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="J43" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="B44" t="s">
-        <v>144</v>
+        <v>211</v>
       </c>
       <c r="C44" t="s">
         <v>11</v>
@@ -3203,30 +3404,30 @@
         <v>11</v>
       </c>
       <c r="E44" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="F44" t="s">
         <v>13</v>
       </c>
       <c r="G44" t="s">
-        <v>146</v>
+        <v>213</v>
       </c>
       <c r="H44" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="I44" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="J44" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="B45" t="s">
-        <v>241</v>
+        <v>211</v>
       </c>
       <c r="C45" t="s">
         <v>11</v>
@@ -3235,30 +3436,30 @@
         <v>11</v>
       </c>
       <c r="E45" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="F45" t="s">
         <v>13</v>
       </c>
       <c r="G45" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="H45" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="I45" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="J45" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="B46" t="s">
-        <v>248</v>
+        <v>211</v>
       </c>
       <c r="C46" t="s">
         <v>11</v>
@@ -3267,30 +3468,30 @@
         <v>11</v>
       </c>
       <c r="E46" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="F46" t="s">
         <v>13</v>
       </c>
       <c r="G46" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="H46" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="I46" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="J46" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="B47" t="s">
-        <v>254</v>
+        <v>211</v>
       </c>
       <c r="C47" t="s">
         <v>11</v>
@@ -3299,30 +3500,30 @@
         <v>11</v>
       </c>
       <c r="E47" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="F47" t="s">
         <v>13</v>
       </c>
       <c r="G47" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="H47" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="I47" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="J47" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="B48" t="s">
-        <v>260</v>
+        <v>211</v>
       </c>
       <c r="C48" t="s">
         <v>11</v>
@@ -3331,30 +3532,30 @@
         <v>11</v>
       </c>
       <c r="E48" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="F48" t="s">
         <v>13</v>
       </c>
       <c r="G48" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="H48" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="I48" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="J48" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B49" t="s">
-        <v>266</v>
+        <v>211</v>
       </c>
       <c r="C49" t="s">
         <v>11</v>
@@ -3363,30 +3564,30 @@
         <v>11</v>
       </c>
       <c r="E49" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F49" t="s">
         <v>13</v>
       </c>
       <c r="G49" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="H49" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="I49" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="J49" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B50" t="s">
-        <v>272</v>
+        <v>211</v>
       </c>
       <c r="C50" t="s">
         <v>11</v>
@@ -3401,7 +3602,7 @@
         <v>13</v>
       </c>
       <c r="G50" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="H50" t="s">
         <v>274</v>
@@ -3418,7 +3619,7 @@
         <v>277</v>
       </c>
       <c r="B51" t="s">
-        <v>260</v>
+        <v>211</v>
       </c>
       <c r="C51" t="s">
         <v>11</v>
@@ -3433,7 +3634,7 @@
         <v>13</v>
       </c>
       <c r="G51" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="H51" t="s">
         <v>279</v>
@@ -3450,455 +3651,455 @@
         <v>282</v>
       </c>
       <c r="B52" t="s">
+        <v>211</v>
+      </c>
+      <c r="C52" t="s">
+        <v>11</v>
+      </c>
+      <c r="D52" t="s">
+        <v>11</v>
+      </c>
+      <c r="E52" t="s">
         <v>283</v>
       </c>
-      <c r="C52" t="s">
-        <v>11</v>
-      </c>
-      <c r="D52" t="s">
-        <v>11</v>
-      </c>
-      <c r="E52" t="s">
+      <c r="F52" t="s">
+        <v>13</v>
+      </c>
+      <c r="G52" t="s">
+        <v>213</v>
+      </c>
+      <c r="H52" t="s">
         <v>284</v>
       </c>
-      <c r="F52" t="s">
-        <v>13</v>
-      </c>
-      <c r="G52" t="s">
-        <v>243</v>
-      </c>
-      <c r="H52" t="s">
+      <c r="I52" t="s">
         <v>285</v>
       </c>
-      <c r="I52" t="s">
+      <c r="J52" t="s">
         <v>286</v>
-      </c>
-      <c r="J52" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>287</v>
+      </c>
+      <c r="B53" t="s">
+        <v>211</v>
+      </c>
+      <c r="C53" t="s">
+        <v>11</v>
+      </c>
+      <c r="D53" t="s">
+        <v>11</v>
+      </c>
+      <c r="E53" t="s">
         <v>288</v>
       </c>
-      <c r="B53" t="s">
+      <c r="F53" t="s">
+        <v>13</v>
+      </c>
+      <c r="G53" t="s">
+        <v>213</v>
+      </c>
+      <c r="H53" t="s">
         <v>289</v>
       </c>
-      <c r="C53" t="s">
-        <v>11</v>
-      </c>
-      <c r="D53" t="s">
-        <v>11</v>
-      </c>
-      <c r="E53" t="s">
+      <c r="I53" t="s">
         <v>290</v>
       </c>
-      <c r="F53" t="s">
-        <v>13</v>
-      </c>
-      <c r="G53" t="s">
-        <v>243</v>
-      </c>
-      <c r="H53" t="s">
+      <c r="J53" t="s">
         <v>291</v>
-      </c>
-      <c r="I53" t="s">
-        <v>292</v>
-      </c>
-      <c r="J53" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>292</v>
+      </c>
+      <c r="B54" t="s">
+        <v>211</v>
+      </c>
+      <c r="C54" t="s">
+        <v>11</v>
+      </c>
+      <c r="D54" t="s">
+        <v>11</v>
+      </c>
+      <c r="E54" t="s">
+        <v>293</v>
+      </c>
+      <c r="F54" t="s">
+        <v>13</v>
+      </c>
+      <c r="G54" t="s">
+        <v>213</v>
+      </c>
+      <c r="H54" t="s">
         <v>294</v>
       </c>
-      <c r="B54" t="s">
+      <c r="I54" t="s">
         <v>295</v>
       </c>
-      <c r="C54" t="s">
-        <v>11</v>
-      </c>
-      <c r="D54" t="s">
-        <v>11</v>
-      </c>
-      <c r="E54" t="s">
+      <c r="J54" t="s">
         <v>296</v>
-      </c>
-      <c r="F54" t="s">
-        <v>13</v>
-      </c>
-      <c r="G54" t="s">
-        <v>243</v>
-      </c>
-      <c r="H54" t="s">
-        <v>297</v>
-      </c>
-      <c r="I54" t="s">
-        <v>298</v>
-      </c>
-      <c r="J54" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>297</v>
+      </c>
+      <c r="B55" t="s">
+        <v>211</v>
+      </c>
+      <c r="C55" t="s">
+        <v>11</v>
+      </c>
+      <c r="D55" t="s">
+        <v>11</v>
+      </c>
+      <c r="E55" t="s">
+        <v>298</v>
+      </c>
+      <c r="F55" t="s">
+        <v>13</v>
+      </c>
+      <c r="G55" t="s">
+        <v>213</v>
+      </c>
+      <c r="H55" t="s">
+        <v>299</v>
+      </c>
+      <c r="I55" t="s">
         <v>300</v>
       </c>
-      <c r="B55" t="s">
+      <c r="J55" t="s">
         <v>301</v>
-      </c>
-      <c r="C55" t="s">
-        <v>11</v>
-      </c>
-      <c r="D55" t="s">
-        <v>11</v>
-      </c>
-      <c r="E55" t="s">
-        <v>302</v>
-      </c>
-      <c r="F55" t="s">
-        <v>13</v>
-      </c>
-      <c r="G55" t="s">
-        <v>243</v>
-      </c>
-      <c r="H55" t="s">
-        <v>303</v>
-      </c>
-      <c r="I55" t="s">
-        <v>304</v>
-      </c>
-      <c r="J55" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>302</v>
+      </c>
+      <c r="B56" t="s">
+        <v>211</v>
+      </c>
+      <c r="C56" t="s">
+        <v>11</v>
+      </c>
+      <c r="D56" t="s">
+        <v>11</v>
+      </c>
+      <c r="E56" t="s">
+        <v>303</v>
+      </c>
+      <c r="F56" t="s">
+        <v>13</v>
+      </c>
+      <c r="G56" t="s">
+        <v>213</v>
+      </c>
+      <c r="H56" t="s">
+        <v>304</v>
+      </c>
+      <c r="I56" t="s">
+        <v>305</v>
+      </c>
+      <c r="J56" t="s">
         <v>306</v>
-      </c>
-      <c r="B56" t="s">
-        <v>307</v>
-      </c>
-      <c r="C56" t="s">
-        <v>11</v>
-      </c>
-      <c r="D56" t="s">
-        <v>11</v>
-      </c>
-      <c r="E56" t="s">
-        <v>308</v>
-      </c>
-      <c r="F56" t="s">
-        <v>13</v>
-      </c>
-      <c r="G56" t="s">
-        <v>243</v>
-      </c>
-      <c r="H56" t="s">
-        <v>309</v>
-      </c>
-      <c r="I56" t="s">
-        <v>310</v>
-      </c>
-      <c r="J56" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>307</v>
+      </c>
+      <c r="B57" t="s">
+        <v>308</v>
+      </c>
+      <c r="C57" t="s">
+        <v>11</v>
+      </c>
+      <c r="D57" t="s">
+        <v>11</v>
+      </c>
+      <c r="E57" t="s">
+        <v>309</v>
+      </c>
+      <c r="F57" t="s">
+        <v>13</v>
+      </c>
+      <c r="G57" t="s">
+        <v>310</v>
+      </c>
+      <c r="H57" t="s">
+        <v>311</v>
+      </c>
+      <c r="I57" t="s">
         <v>312</v>
       </c>
-      <c r="B57" t="s">
-        <v>11</v>
-      </c>
-      <c r="C57" t="s">
+      <c r="J57" t="s">
         <v>313</v>
-      </c>
-      <c r="D57" t="s">
-        <v>314</v>
-      </c>
-      <c r="E57" t="s">
-        <v>315</v>
-      </c>
-      <c r="F57" t="s">
-        <v>316</v>
-      </c>
-      <c r="G57" t="s">
-        <v>11</v>
-      </c>
-      <c r="H57" t="s">
-        <v>317</v>
-      </c>
-      <c r="I57" t="s">
-        <v>11</v>
-      </c>
-      <c r="J57" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>314</v>
+      </c>
+      <c r="B58" t="s">
+        <v>315</v>
+      </c>
+      <c r="C58" t="s">
+        <v>11</v>
+      </c>
+      <c r="D58" t="s">
+        <v>11</v>
+      </c>
+      <c r="E58" t="s">
+        <v>316</v>
+      </c>
+      <c r="F58" t="s">
+        <v>13</v>
+      </c>
+      <c r="G58" t="s">
+        <v>310</v>
+      </c>
+      <c r="H58" t="s">
+        <v>317</v>
+      </c>
+      <c r="I58" t="s">
+        <v>318</v>
+      </c>
+      <c r="J58" t="s">
         <v>319</v>
-      </c>
-      <c r="B58" t="s">
-        <v>320</v>
-      </c>
-      <c r="C58" t="s">
-        <v>11</v>
-      </c>
-      <c r="D58" t="s">
-        <v>11</v>
-      </c>
-      <c r="E58" t="s">
-        <v>321</v>
-      </c>
-      <c r="F58" t="s">
-        <v>13</v>
-      </c>
-      <c r="G58" t="s">
-        <v>243</v>
-      </c>
-      <c r="H58" t="s">
-        <v>322</v>
-      </c>
-      <c r="I58" t="s">
-        <v>323</v>
-      </c>
-      <c r="J58" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>320</v>
+      </c>
+      <c r="B59" t="s">
+        <v>321</v>
+      </c>
+      <c r="C59" t="s">
+        <v>11</v>
+      </c>
+      <c r="D59" t="s">
+        <v>11</v>
+      </c>
+      <c r="E59" t="s">
+        <v>322</v>
+      </c>
+      <c r="F59" t="s">
+        <v>13</v>
+      </c>
+      <c r="G59" t="s">
+        <v>310</v>
+      </c>
+      <c r="H59" t="s">
+        <v>323</v>
+      </c>
+      <c r="I59" t="s">
         <v>324</v>
       </c>
-      <c r="B59" t="s">
+      <c r="J59" t="s">
         <v>325</v>
-      </c>
-      <c r="C59" t="s">
-        <v>11</v>
-      </c>
-      <c r="D59" t="s">
-        <v>11</v>
-      </c>
-      <c r="E59" t="s">
-        <v>326</v>
-      </c>
-      <c r="F59" t="s">
-        <v>13</v>
-      </c>
-      <c r="G59" t="s">
-        <v>327</v>
-      </c>
-      <c r="H59" t="s">
-        <v>328</v>
-      </c>
-      <c r="I59" t="s">
-        <v>329</v>
-      </c>
-      <c r="J59" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>326</v>
+      </c>
+      <c r="B60" t="s">
+        <v>327</v>
+      </c>
+      <c r="C60" t="s">
+        <v>11</v>
+      </c>
+      <c r="D60" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60" t="s">
+        <v>328</v>
+      </c>
+      <c r="F60" t="s">
+        <v>13</v>
+      </c>
+      <c r="G60" t="s">
+        <v>310</v>
+      </c>
+      <c r="H60" t="s">
+        <v>329</v>
+      </c>
+      <c r="I60" t="s">
+        <v>330</v>
+      </c>
+      <c r="J60" t="s">
         <v>331</v>
-      </c>
-      <c r="B60" t="s">
-        <v>325</v>
-      </c>
-      <c r="C60" t="s">
-        <v>11</v>
-      </c>
-      <c r="D60" t="s">
-        <v>11</v>
-      </c>
-      <c r="E60" t="s">
-        <v>332</v>
-      </c>
-      <c r="F60" t="s">
-        <v>13</v>
-      </c>
-      <c r="G60" t="s">
-        <v>327</v>
-      </c>
-      <c r="H60" t="s">
-        <v>333</v>
-      </c>
-      <c r="I60" t="s">
-        <v>334</v>
-      </c>
-      <c r="J60" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>332</v>
+      </c>
+      <c r="B61" t="s">
+        <v>333</v>
+      </c>
+      <c r="C61" t="s">
+        <v>11</v>
+      </c>
+      <c r="D61" t="s">
+        <v>11</v>
+      </c>
+      <c r="E61" t="s">
+        <v>334</v>
+      </c>
+      <c r="F61" t="s">
+        <v>13</v>
+      </c>
+      <c r="G61" t="s">
+        <v>310</v>
+      </c>
+      <c r="H61" t="s">
+        <v>335</v>
+      </c>
+      <c r="I61" t="s">
         <v>336</v>
       </c>
-      <c r="B61" t="s">
-        <v>325</v>
-      </c>
-      <c r="C61" t="s">
-        <v>11</v>
-      </c>
-      <c r="D61" t="s">
-        <v>11</v>
-      </c>
-      <c r="E61" t="s">
+      <c r="J61" t="s">
         <v>337</v>
-      </c>
-      <c r="F61" t="s">
-        <v>13</v>
-      </c>
-      <c r="G61" t="s">
-        <v>327</v>
-      </c>
-      <c r="H61" t="s">
-        <v>338</v>
-      </c>
-      <c r="I61" t="s">
-        <v>339</v>
-      </c>
-      <c r="J61" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>338</v>
+      </c>
+      <c r="B62" t="s">
+        <v>339</v>
+      </c>
+      <c r="C62" t="s">
+        <v>11</v>
+      </c>
+      <c r="D62" t="s">
+        <v>11</v>
+      </c>
+      <c r="E62" t="s">
+        <v>340</v>
+      </c>
+      <c r="F62" t="s">
+        <v>13</v>
+      </c>
+      <c r="G62" t="s">
+        <v>310</v>
+      </c>
+      <c r="H62" t="s">
         <v>341</v>
       </c>
-      <c r="B62" t="s">
-        <v>325</v>
-      </c>
-      <c r="C62" t="s">
-        <v>11</v>
-      </c>
-      <c r="D62" t="s">
-        <v>11</v>
-      </c>
-      <c r="E62" t="s">
+      <c r="I62" t="s">
         <v>342</v>
       </c>
-      <c r="F62" t="s">
-        <v>13</v>
-      </c>
-      <c r="G62" t="s">
-        <v>327</v>
-      </c>
-      <c r="H62" t="s">
+      <c r="J62" t="s">
         <v>343</v>
-      </c>
-      <c r="I62" t="s">
-        <v>344</v>
-      </c>
-      <c r="J62" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>344</v>
+      </c>
+      <c r="B63" t="s">
+        <v>327</v>
+      </c>
+      <c r="C63" t="s">
+        <v>11</v>
+      </c>
+      <c r="D63" t="s">
+        <v>11</v>
+      </c>
+      <c r="E63" t="s">
+        <v>345</v>
+      </c>
+      <c r="F63" t="s">
+        <v>13</v>
+      </c>
+      <c r="G63" t="s">
+        <v>310</v>
+      </c>
+      <c r="H63" t="s">
         <v>346</v>
       </c>
-      <c r="B63" t="s">
-        <v>325</v>
-      </c>
-      <c r="C63" t="s">
-        <v>11</v>
-      </c>
-      <c r="D63" t="s">
-        <v>11</v>
-      </c>
-      <c r="E63" t="s">
+      <c r="I63" t="s">
         <v>347</v>
       </c>
-      <c r="F63" t="s">
-        <v>13</v>
-      </c>
-      <c r="G63" t="s">
-        <v>327</v>
-      </c>
-      <c r="H63" t="s">
+      <c r="J63" t="s">
         <v>348</v>
-      </c>
-      <c r="I63" t="s">
-        <v>349</v>
-      </c>
-      <c r="J63" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>349</v>
+      </c>
+      <c r="B64" t="s">
+        <v>350</v>
+      </c>
+      <c r="C64" t="s">
+        <v>11</v>
+      </c>
+      <c r="D64" t="s">
+        <v>11</v>
+      </c>
+      <c r="E64" t="s">
         <v>351</v>
       </c>
-      <c r="B64" t="s">
-        <v>325</v>
-      </c>
-      <c r="C64" t="s">
-        <v>11</v>
-      </c>
-      <c r="D64" t="s">
-        <v>11</v>
-      </c>
-      <c r="E64" t="s">
+      <c r="F64" t="s">
+        <v>13</v>
+      </c>
+      <c r="G64" t="s">
+        <v>310</v>
+      </c>
+      <c r="H64" t="s">
         <v>352</v>
       </c>
-      <c r="F64" t="s">
-        <v>13</v>
-      </c>
-      <c r="G64" t="s">
-        <v>327</v>
-      </c>
-      <c r="H64" t="s">
+      <c r="I64" t="s">
         <v>353</v>
       </c>
-      <c r="I64" t="s">
+      <c r="J64" t="s">
         <v>354</v>
-      </c>
-      <c r="J64" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>355</v>
+      </c>
+      <c r="B65" t="s">
         <v>356</v>
       </c>
-      <c r="B65" t="s">
+      <c r="C65" t="s">
+        <v>11</v>
+      </c>
+      <c r="D65" t="s">
+        <v>11</v>
+      </c>
+      <c r="E65" t="s">
         <v>357</v>
       </c>
-      <c r="C65" t="s">
-        <v>11</v>
-      </c>
-      <c r="D65" t="s">
-        <v>11</v>
-      </c>
-      <c r="E65" t="s">
+      <c r="F65" t="s">
+        <v>13</v>
+      </c>
+      <c r="G65" t="s">
+        <v>310</v>
+      </c>
+      <c r="H65" t="s">
         <v>358</v>
       </c>
-      <c r="F65" t="s">
-        <v>13</v>
-      </c>
-      <c r="G65" t="s">
-        <v>327</v>
-      </c>
-      <c r="H65" t="s">
+      <c r="I65" t="s">
         <v>359</v>
       </c>
-      <c r="I65" t="s">
+      <c r="J65" t="s">
         <v>360</v>
-      </c>
-      <c r="J65" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>361</v>
+      </c>
+      <c r="B66" t="s">
         <v>362</v>
-      </c>
-      <c r="B66" t="s">
-        <v>325</v>
       </c>
       <c r="C66" t="s">
         <v>11</v>
@@ -3913,7 +4114,7 @@
         <v>13</v>
       </c>
       <c r="G66" t="s">
-        <v>327</v>
+        <v>310</v>
       </c>
       <c r="H66" t="s">
         <v>364</v>
@@ -3945,7 +4146,7 @@
         <v>13</v>
       </c>
       <c r="G67" t="s">
-        <v>327</v>
+        <v>310</v>
       </c>
       <c r="H67" t="s">
         <v>370</v>
@@ -3977,7 +4178,7 @@
         <v>13</v>
       </c>
       <c r="G68" t="s">
-        <v>327</v>
+        <v>310</v>
       </c>
       <c r="H68" t="s">
         <v>376</v>
@@ -3994,71 +4195,71 @@
         <v>379</v>
       </c>
       <c r="B69" t="s">
+        <v>11</v>
+      </c>
+      <c r="C69" t="s">
         <v>380</v>
       </c>
-      <c r="C69" t="s">
-        <v>11</v>
-      </c>
       <c r="D69" t="s">
-        <v>11</v>
+        <v>381</v>
       </c>
       <c r="E69" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F69" t="s">
-        <v>13</v>
+        <v>383</v>
       </c>
       <c r="G69" t="s">
-        <v>327</v>
+        <v>11</v>
       </c>
       <c r="H69" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="I69" t="s">
-        <v>383</v>
+        <v>11</v>
       </c>
       <c r="J69" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>386</v>
+      </c>
+      <c r="B70" t="s">
+        <v>387</v>
+      </c>
+      <c r="C70" t="s">
+        <v>11</v>
+      </c>
+      <c r="D70" t="s">
+        <v>11</v>
+      </c>
+      <c r="E70" t="s">
+        <v>388</v>
+      </c>
+      <c r="F70" t="s">
+        <v>13</v>
+      </c>
+      <c r="G70" t="s">
+        <v>310</v>
+      </c>
+      <c r="H70" t="s">
+        <v>389</v>
+      </c>
+      <c r="I70" t="s">
+        <v>390</v>
+      </c>
+      <c r="J70" t="s">
         <v>385</v>
-      </c>
-      <c r="B70" t="s">
-        <v>325</v>
-      </c>
-      <c r="C70" t="s">
-        <v>11</v>
-      </c>
-      <c r="D70" t="s">
-        <v>11</v>
-      </c>
-      <c r="E70" t="s">
-        <v>386</v>
-      </c>
-      <c r="F70" t="s">
-        <v>13</v>
-      </c>
-      <c r="G70" t="s">
-        <v>327</v>
-      </c>
-      <c r="H70" t="s">
-        <v>387</v>
-      </c>
-      <c r="I70" t="s">
-        <v>388</v>
-      </c>
-      <c r="J70" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B71" t="s">
-        <v>325</v>
+        <v>392</v>
       </c>
       <c r="C71" t="s">
         <v>11</v>
@@ -4067,30 +4268,30 @@
         <v>11</v>
       </c>
       <c r="E71" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="F71" t="s">
         <v>13</v>
       </c>
       <c r="G71" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H71" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="I71" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="J71" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B72" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="C72" t="s">
         <v>11</v>
@@ -4099,30 +4300,30 @@
         <v>11</v>
       </c>
       <c r="E72" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="F72" t="s">
         <v>13</v>
       </c>
       <c r="G72" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H72" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="I72" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="J72" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B73" t="s">
-        <v>380</v>
+        <v>392</v>
       </c>
       <c r="C73" t="s">
         <v>11</v>
@@ -4131,30 +4332,30 @@
         <v>11</v>
       </c>
       <c r="E73" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="F73" t="s">
         <v>13</v>
       </c>
       <c r="G73" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H73" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="I73" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="J73" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B74" t="s">
-        <v>380</v>
+        <v>392</v>
       </c>
       <c r="C74" t="s">
         <v>11</v>
@@ -4163,30 +4364,30 @@
         <v>11</v>
       </c>
       <c r="E74" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="F74" t="s">
         <v>13</v>
       </c>
       <c r="G74" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H74" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="I74" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J74" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B75" t="s">
-        <v>325</v>
+        <v>392</v>
       </c>
       <c r="C75" t="s">
         <v>11</v>
@@ -4195,30 +4396,30 @@
         <v>11</v>
       </c>
       <c r="E75" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="F75" t="s">
         <v>13</v>
       </c>
       <c r="G75" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H75" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="I75" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="J75" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B76" t="s">
-        <v>325</v>
+        <v>392</v>
       </c>
       <c r="C76" t="s">
         <v>11</v>
@@ -4227,30 +4428,30 @@
         <v>11</v>
       </c>
       <c r="E76" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="F76" t="s">
         <v>13</v>
       </c>
       <c r="G76" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H76" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="I76" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="J76" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B77" t="s">
-        <v>325</v>
+        <v>424</v>
       </c>
       <c r="C77" t="s">
         <v>11</v>
@@ -4259,30 +4460,30 @@
         <v>11</v>
       </c>
       <c r="E77" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="F77" t="s">
         <v>13</v>
       </c>
       <c r="G77" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H77" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="I77" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="J77" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="B78" t="s">
-        <v>325</v>
+        <v>392</v>
       </c>
       <c r="C78" t="s">
         <v>11</v>
@@ -4291,30 +4492,30 @@
         <v>11</v>
       </c>
       <c r="E78" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="F78" t="s">
         <v>13</v>
       </c>
       <c r="G78" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H78" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="I78" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="J78" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="B79" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="C79" t="s">
         <v>11</v>
@@ -4323,30 +4524,30 @@
         <v>11</v>
       </c>
       <c r="E79" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="F79" t="s">
         <v>13</v>
       </c>
       <c r="G79" t="s">
-        <v>434</v>
+        <v>394</v>
       </c>
       <c r="H79" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="I79" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="J79" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B80" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C80" t="s">
         <v>11</v>
@@ -4355,30 +4556,30 @@
         <v>11</v>
       </c>
       <c r="E80" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="F80" t="s">
         <v>13</v>
       </c>
       <c r="G80" t="s">
-        <v>441</v>
+        <v>394</v>
       </c>
       <c r="H80" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="I80" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="J80" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B81" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C81" t="s">
         <v>11</v>
@@ -4387,30 +4588,30 @@
         <v>11</v>
       </c>
       <c r="E81" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="F81" t="s">
         <v>13</v>
       </c>
       <c r="G81" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H81" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="I81" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J81" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B82" t="s">
-        <v>452</v>
+        <v>392</v>
       </c>
       <c r="C82" t="s">
         <v>11</v>
@@ -4425,56 +4626,56 @@
         <v>13</v>
       </c>
       <c r="G82" t="s">
+        <v>394</v>
+      </c>
+      <c r="H82" t="s">
         <v>454</v>
       </c>
-      <c r="H82" t="s">
+      <c r="I82" t="s">
         <v>455</v>
       </c>
-      <c r="I82" t="s">
+      <c r="J82" t="s">
         <v>456</v>
-      </c>
-      <c r="J82" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>457</v>
+      </c>
+      <c r="B83" t="s">
+        <v>392</v>
+      </c>
+      <c r="C83" t="s">
+        <v>11</v>
+      </c>
+      <c r="D83" t="s">
+        <v>11</v>
+      </c>
+      <c r="E83" t="s">
         <v>458</v>
       </c>
-      <c r="B83" t="s">
-        <v>325</v>
-      </c>
-      <c r="C83" t="s">
-        <v>11</v>
-      </c>
-      <c r="D83" t="s">
-        <v>11</v>
-      </c>
-      <c r="E83" t="s">
+      <c r="F83" t="s">
+        <v>13</v>
+      </c>
+      <c r="G83" t="s">
+        <v>394</v>
+      </c>
+      <c r="H83" t="s">
         <v>459</v>
       </c>
-      <c r="F83" t="s">
-        <v>13</v>
-      </c>
-      <c r="G83" t="s">
-        <v>327</v>
-      </c>
-      <c r="H83" t="s">
+      <c r="I83" t="s">
         <v>460</v>
       </c>
-      <c r="I83" t="s">
+      <c r="J83" t="s">
         <v>461</v>
-      </c>
-      <c r="J83" t="s">
-        <v>462</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
+        <v>462</v>
+      </c>
+      <c r="B84" t="s">
         <v>463</v>
-      </c>
-      <c r="B84" t="s">
-        <v>446</v>
       </c>
       <c r="C84" t="s">
         <v>11</v>
@@ -4489,7 +4690,7 @@
         <v>13</v>
       </c>
       <c r="G84" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H84" t="s">
         <v>465</v>
@@ -4499,6 +4700,390 @@
       </c>
       <c r="J84" t="s">
         <v>467</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>468</v>
+      </c>
+      <c r="B85" t="s">
+        <v>447</v>
+      </c>
+      <c r="C85" t="s">
+        <v>11</v>
+      </c>
+      <c r="D85" t="s">
+        <v>11</v>
+      </c>
+      <c r="E85" t="s">
+        <v>469</v>
+      </c>
+      <c r="F85" t="s">
+        <v>13</v>
+      </c>
+      <c r="G85" t="s">
+        <v>394</v>
+      </c>
+      <c r="H85" t="s">
+        <v>470</v>
+      </c>
+      <c r="I85" t="s">
+        <v>471</v>
+      </c>
+      <c r="J85" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>473</v>
+      </c>
+      <c r="B86" t="s">
+        <v>447</v>
+      </c>
+      <c r="C86" t="s">
+        <v>11</v>
+      </c>
+      <c r="D86" t="s">
+        <v>11</v>
+      </c>
+      <c r="E86" t="s">
+        <v>474</v>
+      </c>
+      <c r="F86" t="s">
+        <v>13</v>
+      </c>
+      <c r="G86" t="s">
+        <v>394</v>
+      </c>
+      <c r="H86" t="s">
+        <v>475</v>
+      </c>
+      <c r="I86" t="s">
+        <v>476</v>
+      </c>
+      <c r="J86" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>478</v>
+      </c>
+      <c r="B87" t="s">
+        <v>392</v>
+      </c>
+      <c r="C87" t="s">
+        <v>11</v>
+      </c>
+      <c r="D87" t="s">
+        <v>11</v>
+      </c>
+      <c r="E87" t="s">
+        <v>479</v>
+      </c>
+      <c r="F87" t="s">
+        <v>13</v>
+      </c>
+      <c r="G87" t="s">
+        <v>394</v>
+      </c>
+      <c r="H87" t="s">
+        <v>480</v>
+      </c>
+      <c r="I87" t="s">
+        <v>481</v>
+      </c>
+      <c r="J87" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>483</v>
+      </c>
+      <c r="B88" t="s">
+        <v>392</v>
+      </c>
+      <c r="C88" t="s">
+        <v>11</v>
+      </c>
+      <c r="D88" t="s">
+        <v>11</v>
+      </c>
+      <c r="E88" t="s">
+        <v>484</v>
+      </c>
+      <c r="F88" t="s">
+        <v>13</v>
+      </c>
+      <c r="G88" t="s">
+        <v>394</v>
+      </c>
+      <c r="H88" t="s">
+        <v>485</v>
+      </c>
+      <c r="I88" t="s">
+        <v>486</v>
+      </c>
+      <c r="J88" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>488</v>
+      </c>
+      <c r="B89" t="s">
+        <v>392</v>
+      </c>
+      <c r="C89" t="s">
+        <v>11</v>
+      </c>
+      <c r="D89" t="s">
+        <v>11</v>
+      </c>
+      <c r="E89" t="s">
+        <v>489</v>
+      </c>
+      <c r="F89" t="s">
+        <v>13</v>
+      </c>
+      <c r="G89" t="s">
+        <v>394</v>
+      </c>
+      <c r="H89" t="s">
+        <v>490</v>
+      </c>
+      <c r="I89" t="s">
+        <v>491</v>
+      </c>
+      <c r="J89" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>493</v>
+      </c>
+      <c r="B90" t="s">
+        <v>392</v>
+      </c>
+      <c r="C90" t="s">
+        <v>11</v>
+      </c>
+      <c r="D90" t="s">
+        <v>11</v>
+      </c>
+      <c r="E90" t="s">
+        <v>494</v>
+      </c>
+      <c r="F90" t="s">
+        <v>13</v>
+      </c>
+      <c r="G90" t="s">
+        <v>394</v>
+      </c>
+      <c r="H90" t="s">
+        <v>495</v>
+      </c>
+      <c r="I90" t="s">
+        <v>496</v>
+      </c>
+      <c r="J90" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>498</v>
+      </c>
+      <c r="B91" t="s">
+        <v>499</v>
+      </c>
+      <c r="C91" t="s">
+        <v>11</v>
+      </c>
+      <c r="D91" t="s">
+        <v>11</v>
+      </c>
+      <c r="E91" t="s">
+        <v>500</v>
+      </c>
+      <c r="F91" t="s">
+        <v>13</v>
+      </c>
+      <c r="G91" t="s">
+        <v>501</v>
+      </c>
+      <c r="H91" t="s">
+        <v>502</v>
+      </c>
+      <c r="I91" t="s">
+        <v>503</v>
+      </c>
+      <c r="J91" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>505</v>
+      </c>
+      <c r="B92" t="s">
+        <v>506</v>
+      </c>
+      <c r="C92" t="s">
+        <v>11</v>
+      </c>
+      <c r="D92" t="s">
+        <v>11</v>
+      </c>
+      <c r="E92" t="s">
+        <v>507</v>
+      </c>
+      <c r="F92" t="s">
+        <v>13</v>
+      </c>
+      <c r="G92" t="s">
+        <v>508</v>
+      </c>
+      <c r="H92" t="s">
+        <v>509</v>
+      </c>
+      <c r="I92" t="s">
+        <v>510</v>
+      </c>
+      <c r="J92" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>512</v>
+      </c>
+      <c r="B93" t="s">
+        <v>513</v>
+      </c>
+      <c r="C93" t="s">
+        <v>11</v>
+      </c>
+      <c r="D93" t="s">
+        <v>11</v>
+      </c>
+      <c r="E93" t="s">
+        <v>514</v>
+      </c>
+      <c r="F93" t="s">
+        <v>13</v>
+      </c>
+      <c r="G93" t="s">
+        <v>394</v>
+      </c>
+      <c r="H93" t="s">
+        <v>515</v>
+      </c>
+      <c r="I93" t="s">
+        <v>516</v>
+      </c>
+      <c r="J93" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>518</v>
+      </c>
+      <c r="B94" t="s">
+        <v>519</v>
+      </c>
+      <c r="C94" t="s">
+        <v>11</v>
+      </c>
+      <c r="D94" t="s">
+        <v>11</v>
+      </c>
+      <c r="E94" t="s">
+        <v>520</v>
+      </c>
+      <c r="F94" t="s">
+        <v>13</v>
+      </c>
+      <c r="G94" t="s">
+        <v>521</v>
+      </c>
+      <c r="H94" t="s">
+        <v>522</v>
+      </c>
+      <c r="I94" t="s">
+        <v>523</v>
+      </c>
+      <c r="J94" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>525</v>
+      </c>
+      <c r="B95" t="s">
+        <v>392</v>
+      </c>
+      <c r="C95" t="s">
+        <v>11</v>
+      </c>
+      <c r="D95" t="s">
+        <v>11</v>
+      </c>
+      <c r="E95" t="s">
+        <v>526</v>
+      </c>
+      <c r="F95" t="s">
+        <v>13</v>
+      </c>
+      <c r="G95" t="s">
+        <v>394</v>
+      </c>
+      <c r="H95" t="s">
+        <v>527</v>
+      </c>
+      <c r="I95" t="s">
+        <v>528</v>
+      </c>
+      <c r="J95" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>530</v>
+      </c>
+      <c r="B96" t="s">
+        <v>513</v>
+      </c>
+      <c r="C96" t="s">
+        <v>11</v>
+      </c>
+      <c r="D96" t="s">
+        <v>11</v>
+      </c>
+      <c r="E96" t="s">
+        <v>531</v>
+      </c>
+      <c r="F96" t="s">
+        <v>13</v>
+      </c>
+      <c r="G96" t="s">
+        <v>394</v>
+      </c>
+      <c r="H96" t="s">
+        <v>532</v>
+      </c>
+      <c r="I96" t="s">
+        <v>533</v>
+      </c>
+      <c r="J96" t="s">
+        <v>534</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aem 20261011 0826 (#6)
* Add cards-blog, search-blog blocks, update importer

Automated migration updates generated by Experience Modernization Agent.

Changed files: 21

* Add cards-blog, columns-media blocks, update importer

Automated migration updates generated by Experience Modernization Agent.

Changed files: 50

* Update metadata.json

---------

Co-authored-by: AEMY Studio <noreply@aemy.studio>
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-blog-home.report.xlsx
+++ b/tools/importer/reports/import-blog-home.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="535">
   <si>
     <t>_reportFile</t>
   </si>
@@ -349,7 +349,7 @@
     <t>blog-home</t>
   </si>
   <si>
-    <t>2026-10-11T15:20:43.210Z</t>
+    <t>2026-10-11T16:16:44.295Z</t>
   </si>
   <si>
     <t>Blog</t>
@@ -440,6 +440,207 @@
   </si>
   <si>
     <t>https://help.parker.com/us/en/support</t>
+  </si>
+  <si>
+    <t>us/en/blog/comparing-silver-plated-and-nickel-plated-aluminum-emi-shielding-particles.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media"]</t>
+  </si>
+  <si>
+    <t>us/en/blog/comparing-silver-plated-and-nickel-plated-aluminum-emi-shielding-particles</t>
+  </si>
+  <si>
+    <t>blog-article</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:42.179Z</t>
+  </si>
+  <si>
+    <t>Comparing Silver-Plated and Nickel-Plated Aluminum EMI Shielding Particles</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/comparing-silver-plated-and-nickel--plated-aluminum-emi-shielding-particles.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/emi-shielding-and-thermal-management-for-robotics.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media","columns-media","columns-media"]</t>
+  </si>
+  <si>
+    <t>us/en/blog/emi-shielding-and-thermal-management-for-robotics</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:55.942Z</t>
+  </si>
+  <si>
+    <t>EMI Shielding and Thermal Management for Robotics</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/emi-shielding-and-thermal-management-for-robotics.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/emi-shielding-and-thermal-solutions-for-electric-transportation.report.json</t>
+  </si>
+  <si>
+    <t>us/en/blog/emi-shielding-and-thermal-solutions-for-electric-transportation</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:52.773Z</t>
+  </si>
+  <si>
+    <t>EMI Shielding and Thermal Solutions for Electric Transportation</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/emi-shielding-and-thermal-solutions-for-electric-transportation.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/emi-shielding-within-medical-device-applications.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media","columns-media"]</t>
+  </si>
+  <si>
+    <t>us/en/blog/emi-shielding-within-medical-device-applications</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:46.371Z</t>
+  </si>
+  <si>
+    <t>EMI Shielding Within Medical Device Applications</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/emi-shielding-within-medical-device-applications.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/essential-protection-for-high-performance-drone-systems.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media"]</t>
+  </si>
+  <si>
+    <t>us/en/blog/essential-protection-for-high-performance-drone-systems</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:37.529Z</t>
+  </si>
+  <si>
+    <t>EMI Shielding: Essential Protection for High-Performance Drone Systems</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/essential-protection-for-high-performance-drone-systems.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/helping-oems-find-right-hydraulic-cylinder-solution.report.json</t>
+  </si>
+  <si>
+    <t>us/en/blog/helping-oems-find-right-hydraulic-cylinder-solution</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:44.127Z</t>
+  </si>
+  <si>
+    <t>Helping OEMs Find the Right Hydraulic Cylinder Solution</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/msg_grp/helping-oems-find-right-hydraulic-cylinder-solution.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/how-do-thermal-interface-materials-support-leo-small-satellite-electronics.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media","columns-media","columns-media","columns-media","columns-media"]</t>
+  </si>
+  <si>
+    <t>us/en/blog/how-do-thermal-interface-materials-support-leo-small-satellite-electronics</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:39.554Z</t>
+  </si>
+  <si>
+    <t>How Do Thermal Interface Materials Support Low Earth Orbit Small Satellite Electronics</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/how-do-thermal-interface-materials-support-leo-small-satellite-electronics.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/how-parker-chelsea-helps-oems-fleets-improve-pto-performance.report.json</t>
+  </si>
+  <si>
+    <t>us/en/blog/how-parker-chelsea-helps-oems-fleets-improve-pto-performance</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:58.605Z</t>
+  </si>
+  <si>
+    <t>How Parker Chelsea Helps OEMs and Fleets Improve PTO Performance</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/msg_grp/How-Parker-Chelsea-Helps-OEMs-Fleets-Improve-PTO-Performance.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/radar-across-every-domain.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media","table"]</t>
+  </si>
+  <si>
+    <t>us/en/blog/radar-across-every-domain</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:50.925Z</t>
+  </si>
+  <si>
+    <t>Radar Across Every Domain</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/radar-across-every-domain.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/space-payload-emi-shielding.report.json</t>
+  </si>
+  <si>
+    <t>us/en/blog/space-payload-emi-shielding</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:34.973Z</t>
+  </si>
+  <si>
+    <t>Space Payload EMI Shielding: Conductive Gasket Selection for Payload Enclosures</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/space-payload-emi-shielding.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/thermal-management-for-optical-transceivers.report.json</t>
+  </si>
+  <si>
+    <t>us/en/blog/thermal-management-for-optical-transceivers</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:16:00.662Z</t>
+  </si>
+  <si>
+    <t>Thermal Management for Optical Transceivers</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/emg_cho/thermal-management-for-optical-transceivers.html</t>
+  </si>
+  <si>
+    <t>us/en/blog/why-documentation-and-end-user-insight-matter-in-hydraulic-design.report.json</t>
+  </si>
+  <si>
+    <t>us/en/blog/why-documentation-and-end-user-insight-matter-in-hydraulic-design</t>
+  </si>
+  <si>
+    <t>2026-10-11T16:15:48.816Z</t>
+  </si>
+  <si>
+    <t>Why Documentation, Collaboration and End-User Insight Matter in Hydraulic Design</t>
+  </si>
+  <si>
+    <t>https://blog.parker.com/us/en/msg_grp/why-documentation-and-end-user-insight-matter-in-hydraulic-design.html</t>
   </si>
   <si>
     <t>us/en/category/adhesives-coatings-and-encapsulants.report.json</t>
@@ -1805,7 +2006,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J96"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="50" customWidth="1"/>
@@ -2650,7 +2851,7 @@
         <v>150</v>
       </c>
       <c r="B27" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C27" t="s">
         <v>11</v>
@@ -2659,7 +2860,7 @@
         <v>11</v>
       </c>
       <c r="E27" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F27" t="s">
         <v>13</v>
@@ -2668,21 +2869,21 @@
         <v>146</v>
       </c>
       <c r="H27" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I27" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J27" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B28" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C28" t="s">
         <v>11</v>
@@ -2691,7 +2892,7 @@
         <v>11</v>
       </c>
       <c r="E28" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F28" t="s">
         <v>13</v>
@@ -2700,21 +2901,21 @@
         <v>146</v>
       </c>
       <c r="H28" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I28" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J28" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B29" t="s">
-        <v>144</v>
+        <v>162</v>
       </c>
       <c r="C29" t="s">
         <v>11</v>
@@ -2723,7 +2924,7 @@
         <v>11</v>
       </c>
       <c r="E29" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F29" t="s">
         <v>13</v>
@@ -2732,21 +2933,21 @@
         <v>146</v>
       </c>
       <c r="H29" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="I29" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="J29" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B30" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="C30" t="s">
         <v>11</v>
@@ -2755,7 +2956,7 @@
         <v>11</v>
       </c>
       <c r="E30" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="F30" t="s">
         <v>13</v>
@@ -2764,21 +2965,21 @@
         <v>146</v>
       </c>
       <c r="H30" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="I30" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="J30" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B31" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C31" t="s">
         <v>11</v>
@@ -2787,7 +2988,7 @@
         <v>11</v>
       </c>
       <c r="E31" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="F31" t="s">
         <v>13</v>
@@ -2796,21 +2997,21 @@
         <v>146</v>
       </c>
       <c r="H31" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="I31" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="J31" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B32" t="s">
-        <v>144</v>
+        <v>179</v>
       </c>
       <c r="C32" t="s">
         <v>11</v>
@@ -2819,7 +3020,7 @@
         <v>11</v>
       </c>
       <c r="E32" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="F32" t="s">
         <v>13</v>
@@ -2828,21 +3029,21 @@
         <v>146</v>
       </c>
       <c r="H32" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="I32" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="J32" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B33" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C33" t="s">
         <v>11</v>
@@ -2851,7 +3052,7 @@
         <v>11</v>
       </c>
       <c r="E33" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="F33" t="s">
         <v>13</v>
@@ -2860,21 +3061,21 @@
         <v>146</v>
       </c>
       <c r="H33" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="I33" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="J33" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B34" t="s">
-        <v>144</v>
+        <v>190</v>
       </c>
       <c r="C34" t="s">
         <v>11</v>
@@ -2883,7 +3084,7 @@
         <v>11</v>
       </c>
       <c r="E34" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="F34" t="s">
         <v>13</v>
@@ -2892,21 +3093,21 @@
         <v>146</v>
       </c>
       <c r="H34" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="I34" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="J34" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="B35" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C35" t="s">
         <v>11</v>
@@ -2915,7 +3116,7 @@
         <v>11</v>
       </c>
       <c r="E35" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="F35" t="s">
         <v>13</v>
@@ -2924,18 +3125,18 @@
         <v>146</v>
       </c>
       <c r="H35" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="I35" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="J35" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="B36" t="s">
         <v>144</v>
@@ -2947,7 +3148,7 @@
         <v>11</v>
       </c>
       <c r="E36" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="F36" t="s">
         <v>13</v>
@@ -2956,21 +3157,21 @@
         <v>146</v>
       </c>
       <c r="H36" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="I36" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="J36" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="B37" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C37" t="s">
         <v>11</v>
@@ -2979,7 +3180,7 @@
         <v>11</v>
       </c>
       <c r="E37" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="F37" t="s">
         <v>13</v>
@@ -2988,21 +3189,21 @@
         <v>146</v>
       </c>
       <c r="H37" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="I37" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="J37" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="B38" t="s">
-        <v>144</v>
+        <v>211</v>
       </c>
       <c r="C38" t="s">
         <v>11</v>
@@ -3011,30 +3212,30 @@
         <v>11</v>
       </c>
       <c r="E38" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="F38" t="s">
         <v>13</v>
       </c>
       <c r="G38" t="s">
-        <v>146</v>
+        <v>213</v>
       </c>
       <c r="H38" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="I38" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="J38" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="B39" t="s">
-        <v>144</v>
+        <v>211</v>
       </c>
       <c r="C39" t="s">
         <v>11</v>
@@ -3043,30 +3244,30 @@
         <v>11</v>
       </c>
       <c r="E39" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="F39" t="s">
         <v>13</v>
       </c>
       <c r="G39" t="s">
-        <v>146</v>
+        <v>213</v>
       </c>
       <c r="H39" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="I39" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="J39" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="B40" t="s">
-        <v>144</v>
+        <v>211</v>
       </c>
       <c r="C40" t="s">
         <v>11</v>
@@ -3075,30 +3276,30 @@
         <v>11</v>
       </c>
       <c r="E40" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="F40" t="s">
         <v>13</v>
       </c>
       <c r="G40" t="s">
-        <v>146</v>
+        <v>213</v>
       </c>
       <c r="H40" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="I40" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="J40" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="B41" t="s">
-        <v>144</v>
+        <v>211</v>
       </c>
       <c r="C41" t="s">
         <v>11</v>
@@ -3107,30 +3308,30 @@
         <v>11</v>
       </c>
       <c r="E41" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="F41" t="s">
         <v>13</v>
       </c>
       <c r="G41" t="s">
-        <v>146</v>
+        <v>213</v>
       </c>
       <c r="H41" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="I41" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="J41" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="B42" t="s">
-        <v>144</v>
+        <v>211</v>
       </c>
       <c r="C42" t="s">
         <v>11</v>
@@ -3139,30 +3340,30 @@
         <v>11</v>
       </c>
       <c r="E42" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="F42" t="s">
         <v>13</v>
       </c>
       <c r="G42" t="s">
-        <v>146</v>
+        <v>213</v>
       </c>
       <c r="H42" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="I42" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="J42" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="B43" t="s">
-        <v>144</v>
+        <v>211</v>
       </c>
       <c r="C43" t="s">
         <v>11</v>
@@ -3171,30 +3372,30 @@
         <v>11</v>
       </c>
       <c r="E43" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="F43" t="s">
         <v>13</v>
       </c>
       <c r="G43" t="s">
-        <v>146</v>
+        <v>213</v>
       </c>
       <c r="H43" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="I43" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="J43" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="B44" t="s">
-        <v>144</v>
+        <v>211</v>
       </c>
       <c r="C44" t="s">
         <v>11</v>
@@ -3203,30 +3404,30 @@
         <v>11</v>
       </c>
       <c r="E44" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="F44" t="s">
         <v>13</v>
       </c>
       <c r="G44" t="s">
-        <v>146</v>
+        <v>213</v>
       </c>
       <c r="H44" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="I44" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="J44" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="B45" t="s">
-        <v>241</v>
+        <v>211</v>
       </c>
       <c r="C45" t="s">
         <v>11</v>
@@ -3235,30 +3436,30 @@
         <v>11</v>
       </c>
       <c r="E45" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="F45" t="s">
         <v>13</v>
       </c>
       <c r="G45" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="H45" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="I45" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="J45" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="B46" t="s">
-        <v>248</v>
+        <v>211</v>
       </c>
       <c r="C46" t="s">
         <v>11</v>
@@ -3267,30 +3468,30 @@
         <v>11</v>
       </c>
       <c r="E46" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="F46" t="s">
         <v>13</v>
       </c>
       <c r="G46" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="H46" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="I46" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="J46" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="B47" t="s">
-        <v>254</v>
+        <v>211</v>
       </c>
       <c r="C47" t="s">
         <v>11</v>
@@ -3299,30 +3500,30 @@
         <v>11</v>
       </c>
       <c r="E47" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="F47" t="s">
         <v>13</v>
       </c>
       <c r="G47" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="H47" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="I47" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="J47" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="B48" t="s">
-        <v>260</v>
+        <v>211</v>
       </c>
       <c r="C48" t="s">
         <v>11</v>
@@ -3331,30 +3532,30 @@
         <v>11</v>
       </c>
       <c r="E48" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="F48" t="s">
         <v>13</v>
       </c>
       <c r="G48" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="H48" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="I48" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="J48" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B49" t="s">
-        <v>266</v>
+        <v>211</v>
       </c>
       <c r="C49" t="s">
         <v>11</v>
@@ -3363,30 +3564,30 @@
         <v>11</v>
       </c>
       <c r="E49" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F49" t="s">
         <v>13</v>
       </c>
       <c r="G49" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="H49" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="I49" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="J49" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B50" t="s">
-        <v>272</v>
+        <v>211</v>
       </c>
       <c r="C50" t="s">
         <v>11</v>
@@ -3401,7 +3602,7 @@
         <v>13</v>
       </c>
       <c r="G50" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="H50" t="s">
         <v>274</v>
@@ -3418,7 +3619,7 @@
         <v>277</v>
       </c>
       <c r="B51" t="s">
-        <v>260</v>
+        <v>211</v>
       </c>
       <c r="C51" t="s">
         <v>11</v>
@@ -3433,7 +3634,7 @@
         <v>13</v>
       </c>
       <c r="G51" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="H51" t="s">
         <v>279</v>
@@ -3450,455 +3651,455 @@
         <v>282</v>
       </c>
       <c r="B52" t="s">
+        <v>211</v>
+      </c>
+      <c r="C52" t="s">
+        <v>11</v>
+      </c>
+      <c r="D52" t="s">
+        <v>11</v>
+      </c>
+      <c r="E52" t="s">
         <v>283</v>
       </c>
-      <c r="C52" t="s">
-        <v>11</v>
-      </c>
-      <c r="D52" t="s">
-        <v>11</v>
-      </c>
-      <c r="E52" t="s">
+      <c r="F52" t="s">
+        <v>13</v>
+      </c>
+      <c r="G52" t="s">
+        <v>213</v>
+      </c>
+      <c r="H52" t="s">
         <v>284</v>
       </c>
-      <c r="F52" t="s">
-        <v>13</v>
-      </c>
-      <c r="G52" t="s">
-        <v>243</v>
-      </c>
-      <c r="H52" t="s">
+      <c r="I52" t="s">
         <v>285</v>
       </c>
-      <c r="I52" t="s">
+      <c r="J52" t="s">
         <v>286</v>
-      </c>
-      <c r="J52" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>287</v>
+      </c>
+      <c r="B53" t="s">
+        <v>211</v>
+      </c>
+      <c r="C53" t="s">
+        <v>11</v>
+      </c>
+      <c r="D53" t="s">
+        <v>11</v>
+      </c>
+      <c r="E53" t="s">
         <v>288</v>
       </c>
-      <c r="B53" t="s">
+      <c r="F53" t="s">
+        <v>13</v>
+      </c>
+      <c r="G53" t="s">
+        <v>213</v>
+      </c>
+      <c r="H53" t="s">
         <v>289</v>
       </c>
-      <c r="C53" t="s">
-        <v>11</v>
-      </c>
-      <c r="D53" t="s">
-        <v>11</v>
-      </c>
-      <c r="E53" t="s">
+      <c r="I53" t="s">
         <v>290</v>
       </c>
-      <c r="F53" t="s">
-        <v>13</v>
-      </c>
-      <c r="G53" t="s">
-        <v>243</v>
-      </c>
-      <c r="H53" t="s">
+      <c r="J53" t="s">
         <v>291</v>
-      </c>
-      <c r="I53" t="s">
-        <v>292</v>
-      </c>
-      <c r="J53" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>292</v>
+      </c>
+      <c r="B54" t="s">
+        <v>211</v>
+      </c>
+      <c r="C54" t="s">
+        <v>11</v>
+      </c>
+      <c r="D54" t="s">
+        <v>11</v>
+      </c>
+      <c r="E54" t="s">
+        <v>293</v>
+      </c>
+      <c r="F54" t="s">
+        <v>13</v>
+      </c>
+      <c r="G54" t="s">
+        <v>213</v>
+      </c>
+      <c r="H54" t="s">
         <v>294</v>
       </c>
-      <c r="B54" t="s">
+      <c r="I54" t="s">
         <v>295</v>
       </c>
-      <c r="C54" t="s">
-        <v>11</v>
-      </c>
-      <c r="D54" t="s">
-        <v>11</v>
-      </c>
-      <c r="E54" t="s">
+      <c r="J54" t="s">
         <v>296</v>
-      </c>
-      <c r="F54" t="s">
-        <v>13</v>
-      </c>
-      <c r="G54" t="s">
-        <v>243</v>
-      </c>
-      <c r="H54" t="s">
-        <v>297</v>
-      </c>
-      <c r="I54" t="s">
-        <v>298</v>
-      </c>
-      <c r="J54" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>297</v>
+      </c>
+      <c r="B55" t="s">
+        <v>211</v>
+      </c>
+      <c r="C55" t="s">
+        <v>11</v>
+      </c>
+      <c r="D55" t="s">
+        <v>11</v>
+      </c>
+      <c r="E55" t="s">
+        <v>298</v>
+      </c>
+      <c r="F55" t="s">
+        <v>13</v>
+      </c>
+      <c r="G55" t="s">
+        <v>213</v>
+      </c>
+      <c r="H55" t="s">
+        <v>299</v>
+      </c>
+      <c r="I55" t="s">
         <v>300</v>
       </c>
-      <c r="B55" t="s">
+      <c r="J55" t="s">
         <v>301</v>
-      </c>
-      <c r="C55" t="s">
-        <v>11</v>
-      </c>
-      <c r="D55" t="s">
-        <v>11</v>
-      </c>
-      <c r="E55" t="s">
-        <v>302</v>
-      </c>
-      <c r="F55" t="s">
-        <v>13</v>
-      </c>
-      <c r="G55" t="s">
-        <v>243</v>
-      </c>
-      <c r="H55" t="s">
-        <v>303</v>
-      </c>
-      <c r="I55" t="s">
-        <v>304</v>
-      </c>
-      <c r="J55" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>302</v>
+      </c>
+      <c r="B56" t="s">
+        <v>211</v>
+      </c>
+      <c r="C56" t="s">
+        <v>11</v>
+      </c>
+      <c r="D56" t="s">
+        <v>11</v>
+      </c>
+      <c r="E56" t="s">
+        <v>303</v>
+      </c>
+      <c r="F56" t="s">
+        <v>13</v>
+      </c>
+      <c r="G56" t="s">
+        <v>213</v>
+      </c>
+      <c r="H56" t="s">
+        <v>304</v>
+      </c>
+      <c r="I56" t="s">
+        <v>305</v>
+      </c>
+      <c r="J56" t="s">
         <v>306</v>
-      </c>
-      <c r="B56" t="s">
-        <v>307</v>
-      </c>
-      <c r="C56" t="s">
-        <v>11</v>
-      </c>
-      <c r="D56" t="s">
-        <v>11</v>
-      </c>
-      <c r="E56" t="s">
-        <v>308</v>
-      </c>
-      <c r="F56" t="s">
-        <v>13</v>
-      </c>
-      <c r="G56" t="s">
-        <v>243</v>
-      </c>
-      <c r="H56" t="s">
-        <v>309</v>
-      </c>
-      <c r="I56" t="s">
-        <v>310</v>
-      </c>
-      <c r="J56" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>307</v>
+      </c>
+      <c r="B57" t="s">
+        <v>308</v>
+      </c>
+      <c r="C57" t="s">
+        <v>11</v>
+      </c>
+      <c r="D57" t="s">
+        <v>11</v>
+      </c>
+      <c r="E57" t="s">
+        <v>309</v>
+      </c>
+      <c r="F57" t="s">
+        <v>13</v>
+      </c>
+      <c r="G57" t="s">
+        <v>310</v>
+      </c>
+      <c r="H57" t="s">
+        <v>311</v>
+      </c>
+      <c r="I57" t="s">
         <v>312</v>
       </c>
-      <c r="B57" t="s">
-        <v>11</v>
-      </c>
-      <c r="C57" t="s">
+      <c r="J57" t="s">
         <v>313</v>
-      </c>
-      <c r="D57" t="s">
-        <v>314</v>
-      </c>
-      <c r="E57" t="s">
-        <v>315</v>
-      </c>
-      <c r="F57" t="s">
-        <v>316</v>
-      </c>
-      <c r="G57" t="s">
-        <v>11</v>
-      </c>
-      <c r="H57" t="s">
-        <v>317</v>
-      </c>
-      <c r="I57" t="s">
-        <v>11</v>
-      </c>
-      <c r="J57" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>314</v>
+      </c>
+      <c r="B58" t="s">
+        <v>315</v>
+      </c>
+      <c r="C58" t="s">
+        <v>11</v>
+      </c>
+      <c r="D58" t="s">
+        <v>11</v>
+      </c>
+      <c r="E58" t="s">
+        <v>316</v>
+      </c>
+      <c r="F58" t="s">
+        <v>13</v>
+      </c>
+      <c r="G58" t="s">
+        <v>310</v>
+      </c>
+      <c r="H58" t="s">
+        <v>317</v>
+      </c>
+      <c r="I58" t="s">
+        <v>318</v>
+      </c>
+      <c r="J58" t="s">
         <v>319</v>
-      </c>
-      <c r="B58" t="s">
-        <v>320</v>
-      </c>
-      <c r="C58" t="s">
-        <v>11</v>
-      </c>
-      <c r="D58" t="s">
-        <v>11</v>
-      </c>
-      <c r="E58" t="s">
-        <v>321</v>
-      </c>
-      <c r="F58" t="s">
-        <v>13</v>
-      </c>
-      <c r="G58" t="s">
-        <v>243</v>
-      </c>
-      <c r="H58" t="s">
-        <v>322</v>
-      </c>
-      <c r="I58" t="s">
-        <v>323</v>
-      </c>
-      <c r="J58" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>320</v>
+      </c>
+      <c r="B59" t="s">
+        <v>321</v>
+      </c>
+      <c r="C59" t="s">
+        <v>11</v>
+      </c>
+      <c r="D59" t="s">
+        <v>11</v>
+      </c>
+      <c r="E59" t="s">
+        <v>322</v>
+      </c>
+      <c r="F59" t="s">
+        <v>13</v>
+      </c>
+      <c r="G59" t="s">
+        <v>310</v>
+      </c>
+      <c r="H59" t="s">
+        <v>323</v>
+      </c>
+      <c r="I59" t="s">
         <v>324</v>
       </c>
-      <c r="B59" t="s">
+      <c r="J59" t="s">
         <v>325</v>
-      </c>
-      <c r="C59" t="s">
-        <v>11</v>
-      </c>
-      <c r="D59" t="s">
-        <v>11</v>
-      </c>
-      <c r="E59" t="s">
-        <v>326</v>
-      </c>
-      <c r="F59" t="s">
-        <v>13</v>
-      </c>
-      <c r="G59" t="s">
-        <v>327</v>
-      </c>
-      <c r="H59" t="s">
-        <v>328</v>
-      </c>
-      <c r="I59" t="s">
-        <v>329</v>
-      </c>
-      <c r="J59" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>326</v>
+      </c>
+      <c r="B60" t="s">
+        <v>327</v>
+      </c>
+      <c r="C60" t="s">
+        <v>11</v>
+      </c>
+      <c r="D60" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60" t="s">
+        <v>328</v>
+      </c>
+      <c r="F60" t="s">
+        <v>13</v>
+      </c>
+      <c r="G60" t="s">
+        <v>310</v>
+      </c>
+      <c r="H60" t="s">
+        <v>329</v>
+      </c>
+      <c r="I60" t="s">
+        <v>330</v>
+      </c>
+      <c r="J60" t="s">
         <v>331</v>
-      </c>
-      <c r="B60" t="s">
-        <v>325</v>
-      </c>
-      <c r="C60" t="s">
-        <v>11</v>
-      </c>
-      <c r="D60" t="s">
-        <v>11</v>
-      </c>
-      <c r="E60" t="s">
-        <v>332</v>
-      </c>
-      <c r="F60" t="s">
-        <v>13</v>
-      </c>
-      <c r="G60" t="s">
-        <v>327</v>
-      </c>
-      <c r="H60" t="s">
-        <v>333</v>
-      </c>
-      <c r="I60" t="s">
-        <v>334</v>
-      </c>
-      <c r="J60" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>332</v>
+      </c>
+      <c r="B61" t="s">
+        <v>333</v>
+      </c>
+      <c r="C61" t="s">
+        <v>11</v>
+      </c>
+      <c r="D61" t="s">
+        <v>11</v>
+      </c>
+      <c r="E61" t="s">
+        <v>334</v>
+      </c>
+      <c r="F61" t="s">
+        <v>13</v>
+      </c>
+      <c r="G61" t="s">
+        <v>310</v>
+      </c>
+      <c r="H61" t="s">
+        <v>335</v>
+      </c>
+      <c r="I61" t="s">
         <v>336</v>
       </c>
-      <c r="B61" t="s">
-        <v>325</v>
-      </c>
-      <c r="C61" t="s">
-        <v>11</v>
-      </c>
-      <c r="D61" t="s">
-        <v>11</v>
-      </c>
-      <c r="E61" t="s">
+      <c r="J61" t="s">
         <v>337</v>
-      </c>
-      <c r="F61" t="s">
-        <v>13</v>
-      </c>
-      <c r="G61" t="s">
-        <v>327</v>
-      </c>
-      <c r="H61" t="s">
-        <v>338</v>
-      </c>
-      <c r="I61" t="s">
-        <v>339</v>
-      </c>
-      <c r="J61" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>338</v>
+      </c>
+      <c r="B62" t="s">
+        <v>339</v>
+      </c>
+      <c r="C62" t="s">
+        <v>11</v>
+      </c>
+      <c r="D62" t="s">
+        <v>11</v>
+      </c>
+      <c r="E62" t="s">
+        <v>340</v>
+      </c>
+      <c r="F62" t="s">
+        <v>13</v>
+      </c>
+      <c r="G62" t="s">
+        <v>310</v>
+      </c>
+      <c r="H62" t="s">
         <v>341</v>
       </c>
-      <c r="B62" t="s">
-        <v>325</v>
-      </c>
-      <c r="C62" t="s">
-        <v>11</v>
-      </c>
-      <c r="D62" t="s">
-        <v>11</v>
-      </c>
-      <c r="E62" t="s">
+      <c r="I62" t="s">
         <v>342</v>
       </c>
-      <c r="F62" t="s">
-        <v>13</v>
-      </c>
-      <c r="G62" t="s">
-        <v>327</v>
-      </c>
-      <c r="H62" t="s">
+      <c r="J62" t="s">
         <v>343</v>
-      </c>
-      <c r="I62" t="s">
-        <v>344</v>
-      </c>
-      <c r="J62" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>344</v>
+      </c>
+      <c r="B63" t="s">
+        <v>327</v>
+      </c>
+      <c r="C63" t="s">
+        <v>11</v>
+      </c>
+      <c r="D63" t="s">
+        <v>11</v>
+      </c>
+      <c r="E63" t="s">
+        <v>345</v>
+      </c>
+      <c r="F63" t="s">
+        <v>13</v>
+      </c>
+      <c r="G63" t="s">
+        <v>310</v>
+      </c>
+      <c r="H63" t="s">
         <v>346</v>
       </c>
-      <c r="B63" t="s">
-        <v>325</v>
-      </c>
-      <c r="C63" t="s">
-        <v>11</v>
-      </c>
-      <c r="D63" t="s">
-        <v>11</v>
-      </c>
-      <c r="E63" t="s">
+      <c r="I63" t="s">
         <v>347</v>
       </c>
-      <c r="F63" t="s">
-        <v>13</v>
-      </c>
-      <c r="G63" t="s">
-        <v>327</v>
-      </c>
-      <c r="H63" t="s">
+      <c r="J63" t="s">
         <v>348</v>
-      </c>
-      <c r="I63" t="s">
-        <v>349</v>
-      </c>
-      <c r="J63" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>349</v>
+      </c>
+      <c r="B64" t="s">
+        <v>350</v>
+      </c>
+      <c r="C64" t="s">
+        <v>11</v>
+      </c>
+      <c r="D64" t="s">
+        <v>11</v>
+      </c>
+      <c r="E64" t="s">
         <v>351</v>
       </c>
-      <c r="B64" t="s">
-        <v>325</v>
-      </c>
-      <c r="C64" t="s">
-        <v>11</v>
-      </c>
-      <c r="D64" t="s">
-        <v>11</v>
-      </c>
-      <c r="E64" t="s">
+      <c r="F64" t="s">
+        <v>13</v>
+      </c>
+      <c r="G64" t="s">
+        <v>310</v>
+      </c>
+      <c r="H64" t="s">
         <v>352</v>
       </c>
-      <c r="F64" t="s">
-        <v>13</v>
-      </c>
-      <c r="G64" t="s">
-        <v>327</v>
-      </c>
-      <c r="H64" t="s">
+      <c r="I64" t="s">
         <v>353</v>
       </c>
-      <c r="I64" t="s">
+      <c r="J64" t="s">
         <v>354</v>
-      </c>
-      <c r="J64" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>355</v>
+      </c>
+      <c r="B65" t="s">
         <v>356</v>
       </c>
-      <c r="B65" t="s">
+      <c r="C65" t="s">
+        <v>11</v>
+      </c>
+      <c r="D65" t="s">
+        <v>11</v>
+      </c>
+      <c r="E65" t="s">
         <v>357</v>
       </c>
-      <c r="C65" t="s">
-        <v>11</v>
-      </c>
-      <c r="D65" t="s">
-        <v>11</v>
-      </c>
-      <c r="E65" t="s">
+      <c r="F65" t="s">
+        <v>13</v>
+      </c>
+      <c r="G65" t="s">
+        <v>310</v>
+      </c>
+      <c r="H65" t="s">
         <v>358</v>
       </c>
-      <c r="F65" t="s">
-        <v>13</v>
-      </c>
-      <c r="G65" t="s">
-        <v>327</v>
-      </c>
-      <c r="H65" t="s">
+      <c r="I65" t="s">
         <v>359</v>
       </c>
-      <c r="I65" t="s">
+      <c r="J65" t="s">
         <v>360</v>
-      </c>
-      <c r="J65" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>361</v>
+      </c>
+      <c r="B66" t="s">
         <v>362</v>
-      </c>
-      <c r="B66" t="s">
-        <v>325</v>
       </c>
       <c r="C66" t="s">
         <v>11</v>
@@ -3913,7 +4114,7 @@
         <v>13</v>
       </c>
       <c r="G66" t="s">
-        <v>327</v>
+        <v>310</v>
       </c>
       <c r="H66" t="s">
         <v>364</v>
@@ -3945,7 +4146,7 @@
         <v>13</v>
       </c>
       <c r="G67" t="s">
-        <v>327</v>
+        <v>310</v>
       </c>
       <c r="H67" t="s">
         <v>370</v>
@@ -3977,7 +4178,7 @@
         <v>13</v>
       </c>
       <c r="G68" t="s">
-        <v>327</v>
+        <v>310</v>
       </c>
       <c r="H68" t="s">
         <v>376</v>
@@ -3994,71 +4195,71 @@
         <v>379</v>
       </c>
       <c r="B69" t="s">
+        <v>11</v>
+      </c>
+      <c r="C69" t="s">
         <v>380</v>
       </c>
-      <c r="C69" t="s">
-        <v>11</v>
-      </c>
       <c r="D69" t="s">
-        <v>11</v>
+        <v>381</v>
       </c>
       <c r="E69" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F69" t="s">
-        <v>13</v>
+        <v>383</v>
       </c>
       <c r="G69" t="s">
-        <v>327</v>
+        <v>11</v>
       </c>
       <c r="H69" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="I69" t="s">
-        <v>383</v>
+        <v>11</v>
       </c>
       <c r="J69" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>386</v>
+      </c>
+      <c r="B70" t="s">
+        <v>387</v>
+      </c>
+      <c r="C70" t="s">
+        <v>11</v>
+      </c>
+      <c r="D70" t="s">
+        <v>11</v>
+      </c>
+      <c r="E70" t="s">
+        <v>388</v>
+      </c>
+      <c r="F70" t="s">
+        <v>13</v>
+      </c>
+      <c r="G70" t="s">
+        <v>310</v>
+      </c>
+      <c r="H70" t="s">
+        <v>389</v>
+      </c>
+      <c r="I70" t="s">
+        <v>390</v>
+      </c>
+      <c r="J70" t="s">
         <v>385</v>
-      </c>
-      <c r="B70" t="s">
-        <v>325</v>
-      </c>
-      <c r="C70" t="s">
-        <v>11</v>
-      </c>
-      <c r="D70" t="s">
-        <v>11</v>
-      </c>
-      <c r="E70" t="s">
-        <v>386</v>
-      </c>
-      <c r="F70" t="s">
-        <v>13</v>
-      </c>
-      <c r="G70" t="s">
-        <v>327</v>
-      </c>
-      <c r="H70" t="s">
-        <v>387</v>
-      </c>
-      <c r="I70" t="s">
-        <v>388</v>
-      </c>
-      <c r="J70" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B71" t="s">
-        <v>325</v>
+        <v>392</v>
       </c>
       <c r="C71" t="s">
         <v>11</v>
@@ -4067,30 +4268,30 @@
         <v>11</v>
       </c>
       <c r="E71" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="F71" t="s">
         <v>13</v>
       </c>
       <c r="G71" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H71" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="I71" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="J71" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B72" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="C72" t="s">
         <v>11</v>
@@ -4099,30 +4300,30 @@
         <v>11</v>
       </c>
       <c r="E72" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="F72" t="s">
         <v>13</v>
       </c>
       <c r="G72" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H72" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="I72" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="J72" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B73" t="s">
-        <v>380</v>
+        <v>392</v>
       </c>
       <c r="C73" t="s">
         <v>11</v>
@@ -4131,30 +4332,30 @@
         <v>11</v>
       </c>
       <c r="E73" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="F73" t="s">
         <v>13</v>
       </c>
       <c r="G73" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H73" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="I73" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="J73" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B74" t="s">
-        <v>380</v>
+        <v>392</v>
       </c>
       <c r="C74" t="s">
         <v>11</v>
@@ -4163,30 +4364,30 @@
         <v>11</v>
       </c>
       <c r="E74" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="F74" t="s">
         <v>13</v>
       </c>
       <c r="G74" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H74" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="I74" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="J74" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B75" t="s">
-        <v>325</v>
+        <v>392</v>
       </c>
       <c r="C75" t="s">
         <v>11</v>
@@ -4195,30 +4396,30 @@
         <v>11</v>
       </c>
       <c r="E75" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="F75" t="s">
         <v>13</v>
       </c>
       <c r="G75" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H75" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="I75" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="J75" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B76" t="s">
-        <v>325</v>
+        <v>392</v>
       </c>
       <c r="C76" t="s">
         <v>11</v>
@@ -4227,30 +4428,30 @@
         <v>11</v>
       </c>
       <c r="E76" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="F76" t="s">
         <v>13</v>
       </c>
       <c r="G76" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H76" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="I76" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="J76" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B77" t="s">
-        <v>325</v>
+        <v>424</v>
       </c>
       <c r="C77" t="s">
         <v>11</v>
@@ -4259,30 +4460,30 @@
         <v>11</v>
       </c>
       <c r="E77" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="F77" t="s">
         <v>13</v>
       </c>
       <c r="G77" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H77" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="I77" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="J77" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="B78" t="s">
-        <v>325</v>
+        <v>392</v>
       </c>
       <c r="C78" t="s">
         <v>11</v>
@@ -4291,30 +4492,30 @@
         <v>11</v>
       </c>
       <c r="E78" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="F78" t="s">
         <v>13</v>
       </c>
       <c r="G78" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H78" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="I78" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="J78" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="B79" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="C79" t="s">
         <v>11</v>
@@ -4323,30 +4524,30 @@
         <v>11</v>
       </c>
       <c r="E79" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="F79" t="s">
         <v>13</v>
       </c>
       <c r="G79" t="s">
-        <v>434</v>
+        <v>394</v>
       </c>
       <c r="H79" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="I79" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="J79" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B80" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C80" t="s">
         <v>11</v>
@@ -4355,30 +4556,30 @@
         <v>11</v>
       </c>
       <c r="E80" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="F80" t="s">
         <v>13</v>
       </c>
       <c r="G80" t="s">
-        <v>441</v>
+        <v>394</v>
       </c>
       <c r="H80" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="I80" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="J80" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B81" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C81" t="s">
         <v>11</v>
@@ -4387,30 +4588,30 @@
         <v>11</v>
       </c>
       <c r="E81" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="F81" t="s">
         <v>13</v>
       </c>
       <c r="G81" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H81" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="I81" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J81" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B82" t="s">
-        <v>452</v>
+        <v>392</v>
       </c>
       <c r="C82" t="s">
         <v>11</v>
@@ -4425,56 +4626,56 @@
         <v>13</v>
       </c>
       <c r="G82" t="s">
+        <v>394</v>
+      </c>
+      <c r="H82" t="s">
         <v>454</v>
       </c>
-      <c r="H82" t="s">
+      <c r="I82" t="s">
         <v>455</v>
       </c>
-      <c r="I82" t="s">
+      <c r="J82" t="s">
         <v>456</v>
-      </c>
-      <c r="J82" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>457</v>
+      </c>
+      <c r="B83" t="s">
+        <v>392</v>
+      </c>
+      <c r="C83" t="s">
+        <v>11</v>
+      </c>
+      <c r="D83" t="s">
+        <v>11</v>
+      </c>
+      <c r="E83" t="s">
         <v>458</v>
       </c>
-      <c r="B83" t="s">
-        <v>325</v>
-      </c>
-      <c r="C83" t="s">
-        <v>11</v>
-      </c>
-      <c r="D83" t="s">
-        <v>11</v>
-      </c>
-      <c r="E83" t="s">
+      <c r="F83" t="s">
+        <v>13</v>
+      </c>
+      <c r="G83" t="s">
+        <v>394</v>
+      </c>
+      <c r="H83" t="s">
         <v>459</v>
       </c>
-      <c r="F83" t="s">
-        <v>13</v>
-      </c>
-      <c r="G83" t="s">
-        <v>327</v>
-      </c>
-      <c r="H83" t="s">
+      <c r="I83" t="s">
         <v>460</v>
       </c>
-      <c r="I83" t="s">
+      <c r="J83" t="s">
         <v>461</v>
-      </c>
-      <c r="J83" t="s">
-        <v>462</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
+        <v>462</v>
+      </c>
+      <c r="B84" t="s">
         <v>463</v>
-      </c>
-      <c r="B84" t="s">
-        <v>446</v>
       </c>
       <c r="C84" t="s">
         <v>11</v>
@@ -4489,7 +4690,7 @@
         <v>13</v>
       </c>
       <c r="G84" t="s">
-        <v>327</v>
+        <v>394</v>
       </c>
       <c r="H84" t="s">
         <v>465</v>
@@ -4499,6 +4700,390 @@
       </c>
       <c r="J84" t="s">
         <v>467</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>468</v>
+      </c>
+      <c r="B85" t="s">
+        <v>447</v>
+      </c>
+      <c r="C85" t="s">
+        <v>11</v>
+      </c>
+      <c r="D85" t="s">
+        <v>11</v>
+      </c>
+      <c r="E85" t="s">
+        <v>469</v>
+      </c>
+      <c r="F85" t="s">
+        <v>13</v>
+      </c>
+      <c r="G85" t="s">
+        <v>394</v>
+      </c>
+      <c r="H85" t="s">
+        <v>470</v>
+      </c>
+      <c r="I85" t="s">
+        <v>471</v>
+      </c>
+      <c r="J85" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>473</v>
+      </c>
+      <c r="B86" t="s">
+        <v>447</v>
+      </c>
+      <c r="C86" t="s">
+        <v>11</v>
+      </c>
+      <c r="D86" t="s">
+        <v>11</v>
+      </c>
+      <c r="E86" t="s">
+        <v>474</v>
+      </c>
+      <c r="F86" t="s">
+        <v>13</v>
+      </c>
+      <c r="G86" t="s">
+        <v>394</v>
+      </c>
+      <c r="H86" t="s">
+        <v>475</v>
+      </c>
+      <c r="I86" t="s">
+        <v>476</v>
+      </c>
+      <c r="J86" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>478</v>
+      </c>
+      <c r="B87" t="s">
+        <v>392</v>
+      </c>
+      <c r="C87" t="s">
+        <v>11</v>
+      </c>
+      <c r="D87" t="s">
+        <v>11</v>
+      </c>
+      <c r="E87" t="s">
+        <v>479</v>
+      </c>
+      <c r="F87" t="s">
+        <v>13</v>
+      </c>
+      <c r="G87" t="s">
+        <v>394</v>
+      </c>
+      <c r="H87" t="s">
+        <v>480</v>
+      </c>
+      <c r="I87" t="s">
+        <v>481</v>
+      </c>
+      <c r="J87" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>483</v>
+      </c>
+      <c r="B88" t="s">
+        <v>392</v>
+      </c>
+      <c r="C88" t="s">
+        <v>11</v>
+      </c>
+      <c r="D88" t="s">
+        <v>11</v>
+      </c>
+      <c r="E88" t="s">
+        <v>484</v>
+      </c>
+      <c r="F88" t="s">
+        <v>13</v>
+      </c>
+      <c r="G88" t="s">
+        <v>394</v>
+      </c>
+      <c r="H88" t="s">
+        <v>485</v>
+      </c>
+      <c r="I88" t="s">
+        <v>486</v>
+      </c>
+      <c r="J88" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>488</v>
+      </c>
+      <c r="B89" t="s">
+        <v>392</v>
+      </c>
+      <c r="C89" t="s">
+        <v>11</v>
+      </c>
+      <c r="D89" t="s">
+        <v>11</v>
+      </c>
+      <c r="E89" t="s">
+        <v>489</v>
+      </c>
+      <c r="F89" t="s">
+        <v>13</v>
+      </c>
+      <c r="G89" t="s">
+        <v>394</v>
+      </c>
+      <c r="H89" t="s">
+        <v>490</v>
+      </c>
+      <c r="I89" t="s">
+        <v>491</v>
+      </c>
+      <c r="J89" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>493</v>
+      </c>
+      <c r="B90" t="s">
+        <v>392</v>
+      </c>
+      <c r="C90" t="s">
+        <v>11</v>
+      </c>
+      <c r="D90" t="s">
+        <v>11</v>
+      </c>
+      <c r="E90" t="s">
+        <v>494</v>
+      </c>
+      <c r="F90" t="s">
+        <v>13</v>
+      </c>
+      <c r="G90" t="s">
+        <v>394</v>
+      </c>
+      <c r="H90" t="s">
+        <v>495</v>
+      </c>
+      <c r="I90" t="s">
+        <v>496</v>
+      </c>
+      <c r="J90" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>498</v>
+      </c>
+      <c r="B91" t="s">
+        <v>499</v>
+      </c>
+      <c r="C91" t="s">
+        <v>11</v>
+      </c>
+      <c r="D91" t="s">
+        <v>11</v>
+      </c>
+      <c r="E91" t="s">
+        <v>500</v>
+      </c>
+      <c r="F91" t="s">
+        <v>13</v>
+      </c>
+      <c r="G91" t="s">
+        <v>501</v>
+      </c>
+      <c r="H91" t="s">
+        <v>502</v>
+      </c>
+      <c r="I91" t="s">
+        <v>503</v>
+      </c>
+      <c r="J91" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>505</v>
+      </c>
+      <c r="B92" t="s">
+        <v>506</v>
+      </c>
+      <c r="C92" t="s">
+        <v>11</v>
+      </c>
+      <c r="D92" t="s">
+        <v>11</v>
+      </c>
+      <c r="E92" t="s">
+        <v>507</v>
+      </c>
+      <c r="F92" t="s">
+        <v>13</v>
+      </c>
+      <c r="G92" t="s">
+        <v>508</v>
+      </c>
+      <c r="H92" t="s">
+        <v>509</v>
+      </c>
+      <c r="I92" t="s">
+        <v>510</v>
+      </c>
+      <c r="J92" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>512</v>
+      </c>
+      <c r="B93" t="s">
+        <v>513</v>
+      </c>
+      <c r="C93" t="s">
+        <v>11</v>
+      </c>
+      <c r="D93" t="s">
+        <v>11</v>
+      </c>
+      <c r="E93" t="s">
+        <v>514</v>
+      </c>
+      <c r="F93" t="s">
+        <v>13</v>
+      </c>
+      <c r="G93" t="s">
+        <v>394</v>
+      </c>
+      <c r="H93" t="s">
+        <v>515</v>
+      </c>
+      <c r="I93" t="s">
+        <v>516</v>
+      </c>
+      <c r="J93" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>518</v>
+      </c>
+      <c r="B94" t="s">
+        <v>519</v>
+      </c>
+      <c r="C94" t="s">
+        <v>11</v>
+      </c>
+      <c r="D94" t="s">
+        <v>11</v>
+      </c>
+      <c r="E94" t="s">
+        <v>520</v>
+      </c>
+      <c r="F94" t="s">
+        <v>13</v>
+      </c>
+      <c r="G94" t="s">
+        <v>521</v>
+      </c>
+      <c r="H94" t="s">
+        <v>522</v>
+      </c>
+      <c r="I94" t="s">
+        <v>523</v>
+      </c>
+      <c r="J94" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>525</v>
+      </c>
+      <c r="B95" t="s">
+        <v>392</v>
+      </c>
+      <c r="C95" t="s">
+        <v>11</v>
+      </c>
+      <c r="D95" t="s">
+        <v>11</v>
+      </c>
+      <c r="E95" t="s">
+        <v>526</v>
+      </c>
+      <c r="F95" t="s">
+        <v>13</v>
+      </c>
+      <c r="G95" t="s">
+        <v>394</v>
+      </c>
+      <c r="H95" t="s">
+        <v>527</v>
+      </c>
+      <c r="I95" t="s">
+        <v>528</v>
+      </c>
+      <c r="J95" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>530</v>
+      </c>
+      <c r="B96" t="s">
+        <v>513</v>
+      </c>
+      <c r="C96" t="s">
+        <v>11</v>
+      </c>
+      <c r="D96" t="s">
+        <v>11</v>
+      </c>
+      <c r="E96" t="s">
+        <v>531</v>
+      </c>
+      <c r="F96" t="s">
+        <v>13</v>
+      </c>
+      <c r="G96" t="s">
+        <v>394</v>
+      </c>
+      <c r="H96" t="s">
+        <v>532</v>
+      </c>
+      <c r="I96" t="s">
+        <v>533</v>
+      </c>
+      <c r="J96" t="s">
+        <v>534</v>
       </c>
     </row>
   </sheetData>

</xml_diff>